<commit_message>
Update chart of accounts to latest TSCRA COA + account delete button
- Replace COA.xlsx with the new 38-account chart (Direct cost group,
  RHB bank, expenditure codes with 3-digit suffix e.g. 90B1/000)
- Rewrite seed COA to match; accum-depn accounts grouped under assets
- Remap control accounts: INCOME_FEE -> 5000/0001, AP -> 4000/0000
- Update bank/cash labels on reconciliation and cash book pages
- Add delete button for accounts (blocked for control accounts and
  accounts with journal lines, children, or bill references)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/COA.xlsx
+++ b/COA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sharon\Desktop\Accounts\CLIENTS\9. RA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sharon\Desktop\Accounts\CLIENTS\9. RA\2026 TSCRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A2BCEBB-9665-45E1-9C5E-9E7BC25C6E40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{095BA4A7-37B7-4D95-8E7D-29AEB7C6D04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{DF86550E-4A17-4A2D-8989-772EE3724076}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="coa" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="104">
   <si>
     <t>TAMAN SUNWAY CHERAS RESIDENTS ASSOCIATION</t>
   </si>
@@ -45,63 +46,9 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Debit</t>
-  </si>
-  <si>
-    <t>Credit</t>
-  </si>
-  <si>
-    <t>RM</t>
-  </si>
-  <si>
-    <t>1050/000</t>
-  </si>
-  <si>
     <t>Accumulated Fund</t>
   </si>
   <si>
-    <t>2010/000</t>
-  </si>
-  <si>
-    <t>Guard House</t>
-  </si>
-  <si>
-    <t>2010/001</t>
-  </si>
-  <si>
-    <t>Accumulated Depreciation-Guard House</t>
-  </si>
-  <si>
-    <t>2030/000</t>
-  </si>
-  <si>
-    <t>2030/001</t>
-  </si>
-  <si>
-    <t>2040/000</t>
-  </si>
-  <si>
-    <t>Electrical &amp; Fittings</t>
-  </si>
-  <si>
-    <t>2040/001</t>
-  </si>
-  <si>
-    <t>Accumulated Depreciation-Electrical&amp;Ftgs</t>
-  </si>
-  <si>
-    <t>3000/000</t>
-  </si>
-  <si>
-    <t>3010/000</t>
-  </si>
-  <si>
-    <t>RHB Bank</t>
-  </si>
-  <si>
-    <t>3020/000</t>
-  </si>
-  <si>
     <t>Cash</t>
   </si>
   <si>
@@ -126,21 +73,12 @@
     <t>90E1/000</t>
   </si>
   <si>
-    <t>Electricity and water charges</t>
-  </si>
-  <si>
     <t>90G1/000</t>
   </si>
   <si>
     <t>General expenses and maintenance</t>
   </si>
   <si>
-    <t>90M1/000</t>
-  </si>
-  <si>
-    <t>Meeting expenses</t>
-  </si>
-  <si>
     <t>90P1/000</t>
   </si>
   <si>
@@ -159,24 +97,6 @@
     <t>Travelling expenses</t>
   </si>
   <si>
-    <t>Fittings &amp; Signage</t>
-  </si>
-  <si>
-    <t>Accumulated Depreciation-Fittings &amp; Signage</t>
-  </si>
-  <si>
-    <t>2020/000</t>
-  </si>
-  <si>
-    <t>2020/001</t>
-  </si>
-  <si>
-    <t>Amount due from owner units</t>
-  </si>
-  <si>
-    <t>90S1/005</t>
-  </si>
-  <si>
     <t>Services tax</t>
   </si>
   <si>
@@ -189,16 +109,244 @@
     <t>Pond</t>
   </si>
   <si>
-    <t>Accumulated Depreciation-Pond</t>
-  </si>
-  <si>
-    <t>1060/000</t>
-  </si>
-  <si>
-    <t>Retained Earnings</t>
-  </si>
-  <si>
     <t>Chart of accounts</t>
+  </si>
+  <si>
+    <t>Electrical &amp; equipment</t>
+  </si>
+  <si>
+    <t>Fittings &amp; signage</t>
+  </si>
+  <si>
+    <t>Accum depn - Pond</t>
+  </si>
+  <si>
+    <t>Accum depn - Electrical  &amp; equipment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accum depn - Fittings &amp; signage </t>
+  </si>
+  <si>
+    <t>Guard house</t>
+  </si>
+  <si>
+    <t>Accum  depn - Guard house</t>
+  </si>
+  <si>
+    <t>Residents account</t>
+  </si>
+  <si>
+    <t>RHB bank</t>
+  </si>
+  <si>
+    <t>Plant and equipment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classified A/c </t>
+  </si>
+  <si>
+    <t>Group to A/c</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>2000/0000</t>
+  </si>
+  <si>
+    <t>2010/0000</t>
+  </si>
+  <si>
+    <t>2020/0000</t>
+  </si>
+  <si>
+    <t>2030/0000</t>
+  </si>
+  <si>
+    <t>2040/0000</t>
+  </si>
+  <si>
+    <t>3000/0000</t>
+  </si>
+  <si>
+    <t>Deposits and prepayment account</t>
+  </si>
+  <si>
+    <t>3200/0000</t>
+  </si>
+  <si>
+    <t>3300/0000</t>
+  </si>
+  <si>
+    <t>3300/0010</t>
+  </si>
+  <si>
+    <t>4000/0000</t>
+  </si>
+  <si>
+    <t>Payables</t>
+  </si>
+  <si>
+    <t>5000/0000</t>
+  </si>
+  <si>
+    <t>Car stickers</t>
+  </si>
+  <si>
+    <t>TSCRA Membership fee</t>
+  </si>
+  <si>
+    <t>6000/0000</t>
+  </si>
+  <si>
+    <t>INCOME</t>
+  </si>
+  <si>
+    <t>5000/0001</t>
+  </si>
+  <si>
+    <t>5000/0002</t>
+  </si>
+  <si>
+    <t>5000/0003</t>
+  </si>
+  <si>
+    <t>COST OF INCOME</t>
+  </si>
+  <si>
+    <t>6000/0001</t>
+  </si>
+  <si>
+    <t>Security guard services</t>
+  </si>
+  <si>
+    <t>6000/0002</t>
+  </si>
+  <si>
+    <t>6000/0003</t>
+  </si>
+  <si>
+    <t>Security &amp; maintenance</t>
+  </si>
+  <si>
+    <t>CCTV maintenance</t>
+  </si>
+  <si>
+    <t>ADMINISTRATIVE EXPENSES</t>
+  </si>
+  <si>
+    <t>9000/0000</t>
+  </si>
+  <si>
+    <t>Electricity charges</t>
+  </si>
+  <si>
+    <t>Surplus /(deficit) for the year</t>
+  </si>
+  <si>
+    <t>OTHER INCOME</t>
+  </si>
+  <si>
+    <t>Contributions</t>
+  </si>
+  <si>
+    <t>5100/0000</t>
+  </si>
+  <si>
+    <t>5100/0001</t>
+  </si>
+  <si>
+    <t>Balance sheet</t>
+  </si>
+  <si>
+    <t>A/C Type</t>
+  </si>
+  <si>
+    <t>A/c Group</t>
+  </si>
+  <si>
+    <t>Capital &amp; Reserves</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>1000/0000</t>
+  </si>
+  <si>
+    <t>1001/0000</t>
+  </si>
+  <si>
+    <t>Current Assets</t>
+  </si>
+  <si>
+    <t>FA</t>
+  </si>
+  <si>
+    <t>Fixed Assets</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>2010/0100</t>
+  </si>
+  <si>
+    <t>2020/0100</t>
+  </si>
+  <si>
+    <t>2030/0100</t>
+  </si>
+  <si>
+    <t>2040/0100</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Current Liabilities</t>
+  </si>
+  <si>
+    <t>Sundry payables</t>
+  </si>
+  <si>
+    <t>4100/0000</t>
+  </si>
+  <si>
+    <t>Accruals</t>
+  </si>
+  <si>
+    <t>4300/0000</t>
+  </si>
+  <si>
+    <t>DR</t>
+  </si>
+  <si>
+    <t>CR</t>
+  </si>
+  <si>
+    <t>P&amp;L</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Direct cost</t>
+  </si>
+  <si>
+    <t>Expenditure</t>
   </si>
 </sst>
 </file>
@@ -207,9 +355,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="#,###,###,##0.00"/>
+    <numFmt numFmtId="164" formatCode="#,###,###,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -255,6 +403,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -284,16 +453,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -307,7 +474,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -315,13 +482,45 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2 2 2" xfId="3" xr:uid="{95ABBF5F-4AF9-44D1-A401-F41CE2C2593D}"/>
     <cellStyle name="Normal 38" xfId="2" xr:uid="{F7CD2E9E-9A69-4B0F-85A4-EC9BC3CB6988}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -634,15 +833,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACCAE376-6F94-42BB-BE06-07DE381EDC67}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.44140625" style="12" customWidth="1"/>
-    <col min="2" max="2" width="51.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="13.44140625" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="43.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="19.44140625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" style="11" customWidth="1"/>
     <col min="5" max="5" width="17.5546875" customWidth="1"/>
-    <col min="6" max="6" width="13.109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="13.109375" style="24" customWidth="1"/>
     <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="257" max="257" width="15.44140625" customWidth="1"/>
     <col min="258" max="258" width="51.44140625" customWidth="1"/>
@@ -1087,328 +1286,829 @@
     <col min="16136" max="16136" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="F1" s="3"/>
-      <c r="J1" s="3"/>
-    </row>
-    <row r="2" spans="1:10" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="F1" s="25"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" s="1" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A2" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="F2" s="25"/>
+    </row>
+    <row r="3" spans="1:10" s="13" customFormat="1" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="19" t="str">
+        <f>+A5</f>
+        <v>1000/0000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" s="19" t="str">
+        <f>+A6</f>
+        <v>1001/0000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" s="19" t="str">
+        <f t="shared" ref="F7:F8" si="0">+A7</f>
+        <v>2000/0000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F8" s="19" t="str">
+        <f t="shared" si="0"/>
+        <v>2010/0000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="F9" s="19" t="str">
+        <f>+F8</f>
+        <v>2010/0000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" s="19" t="str">
+        <f>+A10</f>
+        <v>2020/0000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="F11" s="19" t="str">
+        <f>+F10</f>
+        <v>2020/0000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F12" s="19" t="str">
+        <f>+A12</f>
+        <v>2030/0000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" s="19" t="str">
+        <f>+F12</f>
+        <v>2030/0000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F14" s="19" t="str">
+        <f>+A14</f>
+        <v>2040/0000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15" s="19" t="str">
+        <f>+F14</f>
+        <v>2040/0000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="F16" s="19" t="str">
+        <f>+A16</f>
+        <v>3000/0000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17" s="20"/>
+      <c r="F17" s="19" t="str">
+        <f>+A17</f>
+        <v>3200/0000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="F18" s="19" t="str">
+        <f>+A18</f>
+        <v>3300/0000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="19" t="str">
+        <f>+A19</f>
+        <v>3300/0010</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="F20" s="19" t="str">
+        <f>+A20</f>
+        <v>4000/0000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="F21" s="19" t="str">
+        <f>+A21</f>
+        <v>4100/0000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C22" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="20"/>
+      <c r="F22" s="19" t="str">
+        <f>+A22</f>
+        <v>4300/0000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="F2" s="3"/>
-    </row>
-    <row r="3" spans="1:10" ht="25.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6" t="s">
+      <c r="C23" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="20"/>
+      <c r="F23" s="19" t="str">
+        <f>+A23</f>
+        <v>5000/0000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="F24" s="19" t="str">
+        <f t="shared" ref="F24:F42" si="1">+A24</f>
+        <v>5000/0001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E25" s="20"/>
+      <c r="F25" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>5000/0002</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" s="20"/>
+      <c r="F26" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>5000/0003</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E27" s="20"/>
+      <c r="F27" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>5100/0000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="E28" s="20"/>
+      <c r="F28" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>5100/0001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" s="20"/>
+      <c r="F29" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>6000/0000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="F30" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>6000/0001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="E31" s="20"/>
+      <c r="F31" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>6000/0002</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32" s="20"/>
+      <c r="F32" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>6000/0003</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="20"/>
+      <c r="F33" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>9000/0000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="B34" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="C34" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E34" s="20"/>
+      <c r="F34" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90B1/000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-    </row>
-    <row r="6" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="B35" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="C35" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E35" s="20"/>
+      <c r="F35" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90C1/000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E36" s="20"/>
+      <c r="F36" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90D1/000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D37" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E37" s="20"/>
+      <c r="F37" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90E1/000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E38" s="20"/>
+      <c r="F38" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90G1/000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="7" t="s">
+      <c r="C39" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D39" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E39" s="8"/>
+      <c r="F39" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90P1/000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
+      <c r="B40" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D40" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E40" s="8"/>
+      <c r="F40" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90S1/000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="7" t="s">
+      <c r="B41" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="7" t="s">
+      <c r="C41" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E41" s="8"/>
+      <c r="F41" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90T1/000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="8" t="s">
+      <c r="B42" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C25" s="9"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-    </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="11"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
+      <c r="C42" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="D42" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="E42" s="8"/>
+      <c r="F42" s="19" t="str">
+        <f t="shared" si="1"/>
+        <v>90U1/000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="10"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="20"/>
+      <c r="E43" s="8"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C44" s="21"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="8"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C45" s="21"/>
+      <c r="D45" s="20"/>
+      <c r="E45" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>